<commit_message>
Kevin: Reestructuración total del sistema de base de datos
</commit_message>
<xml_diff>
--- a/registros_ewaste.xlsx
+++ b/registros_ewaste.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,47 @@
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Destino Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-05-08 10:40:56</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Laptop / Computadora</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>sansum</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>pantalla rota</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>

</xml_diff>